<commit_message>
Add hold exit time calculator
</commit_message>
<xml_diff>
--- a/flow-data/Flow Time Calculator.xlsx
+++ b/flow-data/Flow Time Calculator.xlsx
@@ -5,15 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Cloud Storage\Google Drive\VATSIM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF851F85-0E10-4C6F-B172-C3A4BB802889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{648A068D-5A36-4734-97AD-C9B8440A9CA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="10440" windowWidth="10785" windowHeight="10545" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
-    <sheet name="Calculator" sheetId="8" r:id="rId1"/>
+    <sheet name="Feeder Fix Times" sheetId="8" r:id="rId1"/>
+    <sheet name="Hold Exit Times" sheetId="9" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="FFs">#REF!</definedName>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
   <si>
     <t>From (nm)</t>
   </si>
@@ -74,7 +75,37 @@
     <t>For distances greater than 50nm, reduced speed will incur a +1 minute correction for both jets &amp; non-jets. No correction is required at lesser distances.</t>
   </si>
   <si>
-    <t>.</t>
+    <t>Aircraft</t>
+  </si>
+  <si>
+    <t>Jet</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Distance (nm):</t>
+  </si>
+  <si>
+    <t>KIAS</t>
+  </si>
+  <si>
+    <t>KTAS</t>
+  </si>
+  <si>
+    <t>Reference Data</t>
+  </si>
+  <si>
+    <t>FL140</t>
+  </si>
+  <si>
+    <t>FL200</t>
+  </si>
+  <si>
+    <t>Average Altitude</t>
+  </si>
+  <si>
+    <t>Jet (min):</t>
   </si>
 </sst>
 </file>
@@ -201,7 +232,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -258,6 +289,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -809,7 +843,7 @@
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="19" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C14" s="20"/>
       <c r="D14" s="21"/>
@@ -884,4 +918,131 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{178149F1-5C10-43DF-BEA2-CF4B0A1483C5}">
+  <dimension ref="A2:I24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="9" max="9" width="32.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B2" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="11"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2">
+        <v>210</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="2">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2">
+        <v>250</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="2">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="20"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B17" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" s="18"/>
+      <c r="D17" s="5">
+        <f>E14/E4*60</f>
+        <v>2.3076923076923079</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="13"/>
+      <c r="D18" s="6">
+        <f>E14/E5*60</f>
+        <v>1.7391304347826086</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B23" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="15"/>
+      <c r="I23" s="16"/>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="22"/>
+      <c r="G24" s="22"/>
+      <c r="H24" s="22"/>
+      <c r="I24" s="22"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B24:I24"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B23:I23"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>